<commit_message>
config: atualizar horarios de acesso na planilha
</commit_message>
<xml_diff>
--- a/acessos.xlsx
+++ b/acessos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leonardodel-fhl\Desktop\5. Codigos Python\Projeto Classificação de novos clientes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA01044-2DFA-453E-BC1C-D92726CB2C9A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D956312-BC21-43F1-A261-8D8BA5770C59}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6420" xr2:uid="{15ED11BD-AAF3-4ADB-9705-AF10CDECC0A9}"/>
   </bookViews>
@@ -39,10 +39,10 @@
     <t>horario</t>
   </si>
   <si>
-    <t>qui</t>
-  </si>
-  <si>
-    <t>08:00 - 23:00</t>
+    <t>05:00 - 23:59</t>
+  </si>
+  <si>
+    <t>qui, sex</t>
   </si>
 </sst>
 </file>
@@ -422,10 +422,10 @@
         <v>437112</v>
       </c>
       <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
         <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>